<commit_message>
ML model and solenoid 3d stl added
</commit_message>
<xml_diff>
--- a/Watermelon_Features.xlsx
+++ b/Watermelon_Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mstate-my.sharepoint.com/personal/bm2434_msstate_edu/Documents/Desktop/Watermelon Analysis/Github/Watermelon-Ripeness-Classifier/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_2E899A03D76A1A0E62355476585DCE3A8746D873" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B93AC04-88C7-4826-A20A-0FC9A43F6767}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_2E899A03D76A1A0E62355476585DCE3A8746D873" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8FBA281-C813-4CEE-A264-6B60600300AF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,9 +67,6 @@
     <t>melon1_tap1.wav</t>
   </si>
   <si>
-    <t xml:space="preserve">Ripe </t>
-  </si>
-  <si>
     <t>2026-07-01 16:12:08</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
     <t>melon2_tap1.wav</t>
   </si>
   <si>
-    <t>Overripe</t>
-  </si>
-  <si>
     <t>2026-07-01 17:07:41</t>
   </si>
   <si>
@@ -674,6 +668,12 @@
   </si>
   <si>
     <t>melon9_tap1.wav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ripe </t>
+  </si>
+  <si>
+    <t>overripe</t>
   </si>
 </sst>
 </file>
@@ -1119,12 +1119,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M2" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1133,7 +1133,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>0.24772936105728149</v>
@@ -1160,12 +1160,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M3" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1174,7 +1174,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>0.17534337937831879</v>
@@ -1183,7 +1183,7 @@
         <v>3.0400557443499569E-2</v>
       </c>
       <c r="G4">
-        <v>1.479166666666667E-2</v>
+        <v>1.4791666666666699E-2</v>
       </c>
       <c r="H4">
         <v>-3.0892472706841891</v>
@@ -1201,12 +1201,12 @@
         <v>120</v>
       </c>
       <c r="M4" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1215,7 +1215,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5">
         <v>0.24477848410606379</v>
@@ -1242,12 +1242,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M5" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1256,7 +1256,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6">
         <v>0.20068818330764771</v>
@@ -1283,18 +1283,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M6" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7">
         <v>0.45389235019683838</v>
@@ -1321,18 +1321,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M7" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8">
         <v>0.35128161311149603</v>
@@ -1359,18 +1359,18 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M8" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9">
         <v>0.4684421718120575</v>
@@ -1397,18 +1397,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M9" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10">
         <v>0.53664731979370117</v>
@@ -1435,18 +1435,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M10" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
         <v>32</v>
       </c>
-      <c r="B11" t="s">
-        <v>33</v>
-      </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11">
         <v>0.60924744606018066</v>
@@ -1473,18 +1473,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M11" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
         <v>34</v>
       </c>
-      <c r="B12" t="s">
-        <v>35</v>
-      </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E12">
         <v>0.47143462300300598</v>
@@ -1511,18 +1511,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M12" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
         <v>36</v>
       </c>
-      <c r="B13" t="s">
-        <v>37</v>
-      </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E13">
         <v>0.55836576223373413</v>
@@ -1549,18 +1549,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M13" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
         <v>38</v>
       </c>
-      <c r="B14" t="s">
-        <v>39</v>
-      </c>
       <c r="D14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14">
         <v>0.54909491539001465</v>
@@ -1587,21 +1587,21 @@
         <v>190</v>
       </c>
       <c r="M14" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
         <v>40</v>
-      </c>
-      <c r="B15" t="s">
-        <v>41</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15">
         <v>0.25551652908325201</v>
@@ -1628,21 +1628,21 @@
         <v>103.3333333333333</v>
       </c>
       <c r="M15" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E16">
         <v>0.1397641450166702</v>
@@ -1669,21 +1669,21 @@
         <v>180</v>
       </c>
       <c r="M16" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
       <c r="D17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E17">
         <v>0.25559547543525701</v>
@@ -1710,21 +1710,21 @@
         <v>183.33333333333329</v>
       </c>
       <c r="M17" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>4</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E18">
         <v>0.18200249969959259</v>
@@ -1751,21 +1751,21 @@
         <v>176.66666666666671</v>
       </c>
       <c r="M18" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19">
         <v>5</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>0.25101903080940252</v>
@@ -1792,18 +1792,18 @@
         <v>103.3333333333333</v>
       </c>
       <c r="M19" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E20">
         <v>0.2296462208032608</v>
@@ -1830,18 +1830,18 @@
         <v>100</v>
       </c>
       <c r="M20" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E21">
         <v>0.2145821750164032</v>
@@ -1868,18 +1868,18 @@
         <v>106.6666666666667</v>
       </c>
       <c r="M21" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E22">
         <v>0.1861397325992584</v>
@@ -1906,18 +1906,18 @@
         <v>180</v>
       </c>
       <c r="M22" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E23">
         <v>0.1701568067073822</v>
@@ -1944,18 +1944,18 @@
         <v>180</v>
       </c>
       <c r="M23" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E24">
         <v>0.22825126349925989</v>
@@ -1982,18 +1982,18 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M24" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E25">
         <v>0.18304646015167239</v>
@@ -2020,18 +2020,18 @@
         <v>180</v>
       </c>
       <c r="M25" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D26" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E26">
         <v>0.19856844842433929</v>
@@ -2058,18 +2058,18 @@
         <v>180</v>
       </c>
       <c r="M26" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E27">
         <v>0.26795950531959528</v>
@@ -2096,18 +2096,18 @@
         <v>106.6666666666667</v>
       </c>
       <c r="M27" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E28">
         <v>0.1708436906337738</v>
@@ -2134,18 +2134,18 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M28" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E29">
         <v>0.1914194971323013</v>
@@ -2172,21 +2172,21 @@
         <v>180</v>
       </c>
       <c r="M29" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E30">
         <v>0.79112875461578369</v>
@@ -2213,21 +2213,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M30" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B31" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E31">
         <v>0.74536103010177612</v>
@@ -2254,21 +2254,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M31" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C32">
         <v>2</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E32">
         <v>0.70110964775085449</v>
@@ -2295,21 +2295,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C33">
         <v>3</v>
       </c>
       <c r="D33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E33">
         <v>0.74235647916793823</v>
@@ -2336,21 +2336,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C34">
         <v>4</v>
       </c>
       <c r="D34" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E34">
         <v>0.70704877376556396</v>
@@ -2377,21 +2377,21 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C35">
         <v>5</v>
       </c>
       <c r="D35" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E35">
         <v>0.64414149522781372</v>
@@ -2418,18 +2418,18 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M35" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D36" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E36">
         <v>0.93624967336654663</v>
@@ -2456,18 +2456,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M36" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E37">
         <v>0.69205623865127563</v>
@@ -2494,18 +2494,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E38">
         <v>0.86348420381546021</v>
@@ -2532,18 +2532,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B39" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D39" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E39">
         <v>0.70563942193984985</v>
@@ -2570,18 +2570,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B40" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D40" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E40">
         <v>0.82099103927612305</v>
@@ -2608,18 +2608,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M40" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B41" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E41">
         <v>0.83149176836013794</v>
@@ -2646,18 +2646,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D42" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E42">
         <v>0.71935081481933594</v>
@@ -2684,18 +2684,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M42" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E43">
         <v>0.7887873649597168</v>
@@ -2722,18 +2722,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M43" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D44" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E44">
         <v>0.67659974098205566</v>
@@ -2760,18 +2760,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D45" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E45">
         <v>0.66944444179534912</v>
@@ -2798,18 +2798,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M45" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D46" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E46">
         <v>0.74762886762619019</v>
@@ -2836,18 +2836,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M46" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E47">
         <v>0.67752689123153687</v>
@@ -2874,18 +2874,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M47" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E48">
         <v>0.66052538156509399</v>
@@ -2912,18 +2912,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M48" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B49" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D49" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E49">
         <v>0.57294487953186035</v>
@@ -2950,18 +2950,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M49" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B50" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D50" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E50">
         <v>0.69018644094467163</v>
@@ -2988,21 +2988,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M50" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B51" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C51">
         <v>1</v>
       </c>
       <c r="D51" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E51">
         <v>0.84276449680328369</v>
@@ -3029,12 +3029,12 @@
         <v>200</v>
       </c>
       <c r="M51" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B52">
         <v>4</v>
@@ -3043,7 +3043,7 @@
         <v>2</v>
       </c>
       <c r="D52" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E52">
         <v>0.66242587566375732</v>
@@ -3070,18 +3070,18 @@
         <v>200</v>
       </c>
       <c r="M52" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B53" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D53" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E53">
         <v>0.61060923337936401</v>
@@ -3108,18 +3108,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M53" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E54">
         <v>0.74880105257034302</v>
@@ -3146,18 +3146,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M54" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B55" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D55" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E55">
         <v>0.65678232908248901</v>
@@ -3184,18 +3184,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M55" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B56" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D56" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E56">
         <v>0.44597154855728149</v>
@@ -3222,18 +3222,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M56" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B57" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D57" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E57">
         <v>0.5798267126083374</v>
@@ -3260,18 +3260,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M57" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B58" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D58" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E58">
         <v>0.81914520263671875</v>
@@ -3298,18 +3298,18 @@
         <v>200</v>
       </c>
       <c r="M58" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B59" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D59" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E59">
         <v>0.79886859655380249</v>
@@ -3336,18 +3336,18 @@
         <v>200</v>
       </c>
       <c r="M59" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B60" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D60" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E60">
         <v>0.93908220529556274</v>
@@ -3374,18 +3374,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M60" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B61" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D61" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E61">
         <v>0.69010591506958008</v>
@@ -3412,18 +3412,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M61" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B62" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D62" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E62">
         <v>0.67796504497528076</v>
@@ -3450,21 +3450,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M62" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B63" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C63">
         <v>3</v>
       </c>
       <c r="D63" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E63">
         <v>0.76480108499526978</v>
@@ -3491,21 +3491,21 @@
         <v>200</v>
       </c>
       <c r="M63" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B64" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C64">
         <v>4</v>
       </c>
       <c r="D64" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E64">
         <v>0.74942934513092041</v>
@@ -3532,21 +3532,21 @@
         <v>200</v>
       </c>
       <c r="M64" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B65" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C65">
         <v>5</v>
       </c>
       <c r="D65" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E65">
         <v>0.86284178495407104</v>
@@ -3573,21 +3573,21 @@
         <v>200</v>
       </c>
       <c r="M65" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E66">
         <v>0.73290723562240601</v>
@@ -3614,21 +3614,21 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M66" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B67" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C67">
         <v>2</v>
       </c>
       <c r="D67" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E67">
         <v>0.70988506078720093</v>
@@ -3655,21 +3655,21 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M67" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B68" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C68">
         <v>3</v>
       </c>
       <c r="D68" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E68">
         <v>0.94926232099533081</v>
@@ -3696,21 +3696,21 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M68" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B69" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C69">
         <v>4</v>
       </c>
       <c r="D69" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E69">
         <v>0.72411853075027466</v>
@@ -3737,21 +3737,21 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M69" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B70" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C70">
         <v>5</v>
       </c>
       <c r="D70" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E70">
         <v>0.75415635108947754</v>
@@ -3778,18 +3778,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M70" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B71" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D71" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E71">
         <v>0.94449430704116821</v>
@@ -3816,18 +3816,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M71" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B72" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D72" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E72">
         <v>0.7880101203918457</v>
@@ -3854,18 +3854,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M72" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B73" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D73" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E73">
         <v>0.78574997186660767</v>
@@ -3892,18 +3892,18 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M73" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B74" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D74" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E74">
         <v>0.77242547273635864</v>
@@ -3930,18 +3930,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M74" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B75" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D75" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E75">
         <v>0.77656018733978271</v>
@@ -3968,18 +3968,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M75" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B76" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D76" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E76">
         <v>0.72209632396697998</v>
@@ -4006,18 +4006,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M76" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B77" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D77" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E77">
         <v>0.63622087240219116</v>
@@ -4044,18 +4044,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M77" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B78" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D78" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E78">
         <v>0.49230161309242249</v>
@@ -4082,18 +4082,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M78" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D79" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E79">
         <v>0.55253821611404419</v>
@@ -4120,21 +4120,21 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M79" t="s">
-        <v>15</v>
+        <v>216</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B80" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E80">
         <v>0.61885178089141846</v>
@@ -4161,21 +4161,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M80" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B81" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C81">
         <v>2</v>
       </c>
       <c r="D81" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E81">
         <v>0.65170150995254517</v>
@@ -4202,21 +4202,21 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M81" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B82" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C82">
         <v>3</v>
       </c>
       <c r="D82" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E82">
         <v>0.73112756013870239</v>
@@ -4243,21 +4243,21 @@
         <v>200</v>
       </c>
       <c r="M82" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B83" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C83">
         <v>4</v>
       </c>
       <c r="D83" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E83">
         <v>0.606769859790802</v>
@@ -4284,21 +4284,21 @@
         <v>200</v>
       </c>
       <c r="M83" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B84" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C84">
         <v>5</v>
       </c>
       <c r="D84" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E84">
         <v>0.58059161901473999</v>
@@ -4325,18 +4325,18 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M84" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B85" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D85" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E85">
         <v>0.64421916007995605</v>
@@ -4363,18 +4363,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M85" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B86" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D86" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E86">
         <v>0.65695476531982422</v>
@@ -4401,18 +4401,18 @@
         <v>190</v>
       </c>
       <c r="M86" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B87" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D87" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E87">
         <v>0.61346125602722168</v>
@@ -4439,18 +4439,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M87" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B88" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D88" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E88">
         <v>0.60480892658233643</v>
@@ -4477,18 +4477,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M88" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B89" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D89" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E89">
         <v>0.59211194515228271</v>
@@ -4515,18 +4515,18 @@
         <v>180</v>
       </c>
       <c r="M89" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B90" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D90" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E90">
         <v>0.76281583309173584</v>
@@ -4553,18 +4553,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M90" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B91" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D91" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E91">
         <v>0.7515333890914917</v>
@@ -4591,18 +4591,18 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M91" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B92" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D92" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E92">
         <v>0.5477796196937561</v>
@@ -4629,18 +4629,18 @@
         <v>200</v>
       </c>
       <c r="M92" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B93" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D93" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E93">
         <v>0.63564527034759521</v>
@@ -4667,18 +4667,18 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M93" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B94" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D94" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E94">
         <v>0.59530627727508545</v>
@@ -4705,21 +4705,21 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M94" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B95" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C95">
         <v>1</v>
       </c>
       <c r="D95" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E95">
         <v>0.38947203755378718</v>
@@ -4746,21 +4746,21 @@
         <v>140</v>
       </c>
       <c r="M95" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B96" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C96">
         <v>2</v>
       </c>
       <c r="D96" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E96">
         <v>0.36370760202407842</v>
@@ -4787,21 +4787,21 @@
         <v>120</v>
       </c>
       <c r="M96" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B97" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C97">
         <v>1</v>
       </c>
       <c r="D97" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E97">
         <v>0.2409983575344086</v>
@@ -4828,21 +4828,21 @@
         <v>120</v>
       </c>
       <c r="M97" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
+        <v>212</v>
+      </c>
+      <c r="B98" t="s">
+        <v>213</v>
+      </c>
+      <c r="C98" t="s">
         <v>214</v>
       </c>
-      <c r="B98" t="s">
+      <c r="D98" t="s">
         <v>215</v>
-      </c>
-      <c r="C98" t="s">
-        <v>216</v>
-      </c>
-      <c r="D98" t="s">
-        <v>217</v>
       </c>
       <c r="E98">
         <v>0.79560792446136475</v>
@@ -4869,10 +4869,11 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M98" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ML code samples added for testing
</commit_message>
<xml_diff>
--- a/Watermelon_Features.xlsx
+++ b/Watermelon_Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mstate-my.sharepoint.com/personal/bm2434_msstate_edu/Documents/Desktop/Watermelon Analysis/Github/Watermelon-Ripeness-Classifier/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_2E899A03D76A1A0E62355476585DCE3A8746D873" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8FBA281-C813-4CEE-A264-6B60600300AF}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="11_2E899A03D76A1A0E62355476585DCE3A8746D873" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAF980A3-C742-4223-9714-502B5589D918}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,18 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="218">
-  <si>
-    <t>timestamp</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="23">
   <si>
     <t>melon_id</t>
   </si>
   <si>
     <t>tap_id</t>
-  </si>
-  <si>
-    <t>source_file</t>
   </si>
   <si>
     <t>peak_amplitude</t>
@@ -61,613 +55,34 @@
     <t>LABEL</t>
   </si>
   <si>
-    <t>2026-07-01 16:11:38</t>
-  </si>
-  <si>
-    <t>melon1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:12:08</t>
-  </si>
-  <si>
-    <t>melon1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:12:59</t>
-  </si>
-  <si>
-    <t>melon1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:13:20</t>
-  </si>
-  <si>
-    <t>melon1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:13:32</t>
-  </si>
-  <si>
-    <t>melon1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:48:45</t>
-  </si>
-  <si>
-    <t>melon1.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:49:17</t>
-  </si>
-  <si>
-    <t>melon1.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 16:50:04</t>
-  </si>
-  <si>
-    <t>melon1.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:01:43</t>
-  </si>
-  <si>
-    <t>melon1.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:02:08</t>
-  </si>
-  <si>
-    <t>melon1.2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:02:21</t>
-  </si>
-  <si>
-    <t>melon1.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:02:34</t>
-  </si>
-  <si>
-    <t>melon1.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:02:49</t>
-  </si>
-  <si>
-    <t>melon1.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:07:13</t>
-  </si>
-  <si>
     <t>2</t>
-  </si>
-  <si>
-    <t>melon2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:07:41</t>
-  </si>
-  <si>
-    <t>melon2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:08:02</t>
-  </si>
-  <si>
-    <t>melon2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:08:29</t>
-  </si>
-  <si>
-    <t>melon2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:08:46</t>
-  </si>
-  <si>
-    <t>melon2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:09:09</t>
-  </si>
-  <si>
-    <t>melon2.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:12:26</t>
-  </si>
-  <si>
-    <t>melon2.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:12:39</t>
-  </si>
-  <si>
-    <t>melon2.1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:12:54</t>
-  </si>
-  <si>
-    <t>melon2.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:13:12</t>
-  </si>
-  <si>
-    <t>melon2.1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:13:33</t>
-  </si>
-  <si>
-    <t>melon2.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:13:47</t>
-  </si>
-  <si>
-    <t>melon2.2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:14:01</t>
-  </si>
-  <si>
-    <t>melon2.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:14:13</t>
-  </si>
-  <si>
-    <t>melon2.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-01 17:14:26</t>
-  </si>
-  <si>
-    <t>melon2.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:54:56</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
-    <t>melon3_tap1.wav</t>
-  </si>
-  <si>
     <t>unripe</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:56:41</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:56:52</t>
-  </si>
-  <si>
-    <t>melon3_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:57:45</t>
-  </si>
-  <si>
-    <t>melon3_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:57:59</t>
-  </si>
-  <si>
-    <t>melon3_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 12:58:22</t>
-  </si>
-  <si>
-    <t>melon3_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:01:13</t>
-  </si>
-  <si>
-    <t>melon3.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:01:43</t>
-  </si>
-  <si>
-    <t>melon3.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:01:58</t>
-  </si>
-  <si>
-    <t>melon3.1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:02:23</t>
-  </si>
-  <si>
-    <t>melon3.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:02:36</t>
-  </si>
-  <si>
-    <t>melon3.1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:05:22</t>
-  </si>
-  <si>
-    <t>melon3.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:05:44</t>
-  </si>
-  <si>
-    <t>melon3.2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:06:02</t>
-  </si>
-  <si>
-    <t>melon3.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:06:17</t>
-  </si>
-  <si>
-    <t>melon3.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:06:42</t>
-  </si>
-  <si>
-    <t>melon3.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:13:46</t>
-  </si>
-  <si>
-    <t>melon3.3_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:14:02</t>
-  </si>
-  <si>
-    <t>melon3.3_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:14:17</t>
-  </si>
-  <si>
-    <t>melon3.3_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:15:04</t>
-  </si>
-  <si>
-    <t>melon3.3_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:15:16</t>
-  </si>
-  <si>
-    <t>melon3.3_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:27:21</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>melon4_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:28:05</t>
-  </si>
-  <si>
-    <t>melon4_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:31:16</t>
-  </si>
-  <si>
-    <t>melon4.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:33:07</t>
-  </si>
-  <si>
-    <t>melon4.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:33:18</t>
-  </si>
-  <si>
-    <t>melon4.1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:33:34</t>
-  </si>
-  <si>
-    <t>melon4.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:33:48</t>
-  </si>
-  <si>
-    <t>melon4.1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:37:57</t>
-  </si>
-  <si>
-    <t>melon4.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:38:09</t>
-  </si>
-  <si>
-    <t>melon4.2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:38:22</t>
-  </si>
-  <si>
-    <t>melon4.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:38:37</t>
-  </si>
-  <si>
-    <t>melon4.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:38:50</t>
-  </si>
-  <si>
-    <t>melon4.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:49:10</t>
-  </si>
-  <si>
-    <t>melon4_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:49:21</t>
-  </si>
-  <si>
-    <t>melon4_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 13:49:36</t>
-  </si>
-  <si>
-    <t>melon4_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:03:51</t>
-  </si>
-  <si>
     <t>5</t>
-  </si>
-  <si>
-    <t>melon5_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:04:10</t>
-  </si>
-  <si>
-    <t>melon5_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:04:21</t>
-  </si>
-  <si>
-    <t>melon5_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:05:05</t>
-  </si>
-  <si>
-    <t>melon5_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:05:15</t>
-  </si>
-  <si>
-    <t>melon5_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:05:29</t>
-  </si>
-  <si>
-    <t>melon5.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:05:40</t>
-  </si>
-  <si>
-    <t>melon5.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:05:50</t>
-  </si>
-  <si>
-    <t>melon5.1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:06:00</t>
-  </si>
-  <si>
-    <t>melon5.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:06:29</t>
-  </si>
-  <si>
-    <t>melon5.1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:06:40</t>
-  </si>
-  <si>
-    <t>melon5.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:07:02</t>
-  </si>
-  <si>
-    <t>melon5.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:07:13</t>
-  </si>
-  <si>
-    <t>melon5.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:07:25</t>
-  </si>
-  <si>
-    <t>melon5.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:15:03</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t>melon6_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:15:29</t>
-  </si>
-  <si>
-    <t>melon6_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:19:14</t>
-  </si>
-  <si>
-    <t>melon6_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:19:39</t>
-  </si>
-  <si>
-    <t>melon6_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:19:52</t>
-  </si>
-  <si>
-    <t>melon6_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:20:08</t>
-  </si>
-  <si>
-    <t>melon6.1_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:20:18</t>
-  </si>
-  <si>
-    <t>melon6.1_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:20:43</t>
-  </si>
-  <si>
-    <t>melon6.1_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:20:54</t>
-  </si>
-  <si>
-    <t>melon6.1_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:21:04</t>
-  </si>
-  <si>
-    <t>melon6.1_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:21:26</t>
-  </si>
-  <si>
-    <t>melon6.2_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:21:38</t>
-  </si>
-  <si>
-    <t>melon6.2_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:21:49</t>
-  </si>
-  <si>
-    <t>melon6.2_tap3.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:22:00</t>
-  </si>
-  <si>
-    <t>melon6.2_tap4.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:22:16</t>
-  </si>
-  <si>
-    <t>melon6.2_tap5.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:24:55</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
-    <t>melon7_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:25:08</t>
-  </si>
-  <si>
-    <t>melon7_tap2.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 14:50:34</t>
-  </si>
-  <si>
     <t>8</t>
-  </si>
-  <si>
-    <t>melon8_tap1.wav</t>
-  </si>
-  <si>
-    <t>2026-07-02 15:04:13</t>
   </si>
   <si>
     <t>9</t>
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>melon9_tap1.wav</t>
   </si>
   <si>
     <t xml:space="preserve">ripe </t>
@@ -1038,62 +453,66 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="17.77734375" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.88671875" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" customWidth="1"/>
+    <col min="10" max="10" width="22.21875" customWidth="1"/>
+    <col min="11" max="11" width="15.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1"/>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="N1" s="1"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
       <c r="E2">
         <v>0.1854978799819946</v>
       </c>
@@ -1119,22 +538,16 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M2" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
       <c r="E3">
         <v>0.24772936105728149</v>
       </c>
@@ -1160,22 +573,16 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M3" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
       <c r="E4">
         <v>0.17534337937831879</v>
       </c>
@@ -1201,22 +608,16 @@
         <v>120</v>
       </c>
       <c r="M4" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
       <c r="E5">
         <v>0.24477848410606379</v>
       </c>
@@ -1242,22 +643,16 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M5" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
       <c r="E6">
         <v>0.20068818330764771</v>
       </c>
@@ -1283,18 +678,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M6" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
       </c>
       <c r="E7">
         <v>0.45389235019683838</v>
@@ -1321,18 +713,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M7" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
       </c>
       <c r="E8">
         <v>0.35128161311149603</v>
@@ -1359,18 +748,15 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M8" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
       </c>
       <c r="E9">
         <v>0.4684421718120575</v>
@@ -1397,18 +783,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M9" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>30</v>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
       </c>
       <c r="E10">
         <v>0.53664731979370117</v>
@@ -1435,18 +818,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M10" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>32</v>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
       </c>
       <c r="E11">
         <v>0.60924744606018066</v>
@@ -1473,18 +853,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M11" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" t="s">
-        <v>34</v>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>11</v>
       </c>
       <c r="E12">
         <v>0.47143462300300598</v>
@@ -1511,18 +888,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M12" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>36</v>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>12</v>
       </c>
       <c r="E13">
         <v>0.55836576223373413</v>
@@ -1549,18 +923,15 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M13" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>13</v>
       </c>
       <c r="E14">
         <v>0.54909491539001465</v>
@@ -1587,22 +958,16 @@
         <v>190</v>
       </c>
       <c r="M14" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>39</v>
-      </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" t="s">
-        <v>41</v>
-      </c>
       <c r="E15">
         <v>0.25551652908325201</v>
       </c>
@@ -1628,22 +993,16 @@
         <v>103.3333333333333</v>
       </c>
       <c r="M15" t="s">
-        <v>217</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>42</v>
-      </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16" t="s">
-        <v>43</v>
-      </c>
       <c r="E16">
         <v>0.1397641450166702</v>
       </c>
@@ -1669,22 +1028,16 @@
         <v>180</v>
       </c>
       <c r="M16" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>44</v>
-      </c>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
-      <c r="D17" t="s">
-        <v>45</v>
-      </c>
       <c r="E17">
         <v>0.25559547543525701</v>
       </c>
@@ -1710,22 +1063,16 @@
         <v>183.33333333333329</v>
       </c>
       <c r="M17" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>46</v>
-      </c>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C18">
         <v>4</v>
       </c>
-      <c r="D18" t="s">
-        <v>47</v>
-      </c>
       <c r="E18">
         <v>0.18200249969959259</v>
       </c>
@@ -1751,22 +1098,16 @@
         <v>176.66666666666671</v>
       </c>
       <c r="M18" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>48</v>
-      </c>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C19">
         <v>5</v>
       </c>
-      <c r="D19" t="s">
-        <v>49</v>
-      </c>
       <c r="E19">
         <v>0.25101903080940252</v>
       </c>
@@ -1792,18 +1133,12 @@
         <v>103.3333333333333</v>
       </c>
       <c r="M19" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" t="s">
-        <v>51</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>2</v>
       </c>
       <c r="E20">
         <v>0.2296462208032608</v>
@@ -1830,18 +1165,12 @@
         <v>100</v>
       </c>
       <c r="M20" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" t="s">
-        <v>53</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <v>2</v>
       </c>
       <c r="E21">
         <v>0.2145821750164032</v>
@@ -1868,18 +1197,12 @@
         <v>106.6666666666667</v>
       </c>
       <c r="M21" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" t="s">
-        <v>55</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>2</v>
       </c>
       <c r="E22">
         <v>0.1861397325992584</v>
@@ -1906,18 +1229,12 @@
         <v>180</v>
       </c>
       <c r="M22" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" t="s">
-        <v>57</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>2</v>
       </c>
       <c r="E23">
         <v>0.1701568067073822</v>
@@ -1944,18 +1261,12 @@
         <v>180</v>
       </c>
       <c r="M23" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" t="s">
-        <v>59</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>2</v>
       </c>
       <c r="E24">
         <v>0.22825126349925989</v>
@@ -1982,18 +1293,12 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M24" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" t="s">
-        <v>61</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>2</v>
       </c>
       <c r="E25">
         <v>0.18304646015167239</v>
@@ -2020,18 +1325,12 @@
         <v>180</v>
       </c>
       <c r="M25" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>62</v>
-      </c>
-      <c r="B26" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" t="s">
-        <v>63</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <v>2</v>
       </c>
       <c r="E26">
         <v>0.19856844842433929</v>
@@ -2058,18 +1357,12 @@
         <v>180</v>
       </c>
       <c r="M26" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>64</v>
-      </c>
-      <c r="B27" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" t="s">
-        <v>65</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B27">
+        <v>2</v>
       </c>
       <c r="E27">
         <v>0.26795950531959528</v>
@@ -2096,18 +1389,12 @@
         <v>106.6666666666667</v>
       </c>
       <c r="M27" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B28" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" t="s">
-        <v>67</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B28">
+        <v>2</v>
       </c>
       <c r="E28">
         <v>0.1708436906337738</v>
@@ -2134,18 +1421,12 @@
         <v>186.66666666666671</v>
       </c>
       <c r="M28" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>68</v>
-      </c>
-      <c r="B29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" t="s">
-        <v>69</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <v>2</v>
       </c>
       <c r="E29">
         <v>0.1914194971323013</v>
@@ -2172,22 +1453,16 @@
         <v>180</v>
       </c>
       <c r="M29" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>70</v>
-      </c>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
-      <c r="D30" t="s">
-        <v>72</v>
-      </c>
       <c r="E30">
         <v>0.79112875461578369</v>
       </c>
@@ -2213,22 +1488,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M30" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>74</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
-      <c r="D31" t="s">
-        <v>72</v>
-      </c>
       <c r="E31">
         <v>0.74536103010177612</v>
       </c>
@@ -2254,22 +1523,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M31" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>75</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C32">
         <v>2</v>
       </c>
-      <c r="D32" t="s">
-        <v>76</v>
-      </c>
       <c r="E32">
         <v>0.70110964775085449</v>
       </c>
@@ -2295,22 +1558,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M32" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>77</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C33">
         <v>3</v>
       </c>
-      <c r="D33" t="s">
-        <v>78</v>
-      </c>
       <c r="E33">
         <v>0.74235647916793823</v>
       </c>
@@ -2336,22 +1593,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M33" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>79</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C34">
         <v>4</v>
       </c>
-      <c r="D34" t="s">
-        <v>80</v>
-      </c>
       <c r="E34">
         <v>0.70704877376556396</v>
       </c>
@@ -2377,22 +1628,16 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M34" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>81</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C35">
         <v>5</v>
       </c>
-      <c r="D35" t="s">
-        <v>82</v>
-      </c>
       <c r="E35">
         <v>0.64414149522781372</v>
       </c>
@@ -2418,18 +1663,12 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M35" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>83</v>
-      </c>
-      <c r="B36" t="s">
-        <v>84</v>
-      </c>
-      <c r="D36" t="s">
-        <v>84</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B36">
+        <v>3</v>
       </c>
       <c r="E36">
         <v>0.93624967336654663</v>
@@ -2456,18 +1695,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M36" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>85</v>
-      </c>
-      <c r="B37" t="s">
-        <v>86</v>
-      </c>
-      <c r="D37" t="s">
-        <v>86</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <v>3</v>
       </c>
       <c r="E37">
         <v>0.69205623865127563</v>
@@ -2494,18 +1727,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M37" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>87</v>
-      </c>
-      <c r="B38" t="s">
-        <v>88</v>
-      </c>
-      <c r="D38" t="s">
-        <v>88</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B38">
+        <v>3</v>
       </c>
       <c r="E38">
         <v>0.86348420381546021</v>
@@ -2532,18 +1759,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M38" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>89</v>
-      </c>
-      <c r="B39" t="s">
-        <v>90</v>
-      </c>
-      <c r="D39" t="s">
-        <v>90</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B39">
+        <v>3</v>
       </c>
       <c r="E39">
         <v>0.70563942193984985</v>
@@ -2570,18 +1791,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M39" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>91</v>
-      </c>
-      <c r="B40" t="s">
-        <v>92</v>
-      </c>
-      <c r="D40" t="s">
-        <v>92</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B40">
+        <v>3</v>
       </c>
       <c r="E40">
         <v>0.82099103927612305</v>
@@ -2608,18 +1823,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M40" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" t="s">
-        <v>94</v>
-      </c>
-      <c r="D41" t="s">
-        <v>94</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B41">
+        <v>3</v>
       </c>
       <c r="E41">
         <v>0.83149176836013794</v>
@@ -2646,18 +1855,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M41" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>95</v>
-      </c>
-      <c r="B42" t="s">
-        <v>96</v>
-      </c>
-      <c r="D42" t="s">
-        <v>96</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B42">
+        <v>3</v>
       </c>
       <c r="E42">
         <v>0.71935081481933594</v>
@@ -2684,18 +1887,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M42" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>97</v>
-      </c>
-      <c r="B43" t="s">
-        <v>98</v>
-      </c>
-      <c r="D43" t="s">
-        <v>98</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>3</v>
       </c>
       <c r="E43">
         <v>0.7887873649597168</v>
@@ -2722,18 +1919,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M43" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>99</v>
-      </c>
-      <c r="B44" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" t="s">
-        <v>100</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B44">
+        <v>3</v>
       </c>
       <c r="E44">
         <v>0.67659974098205566</v>
@@ -2760,18 +1951,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M44" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>101</v>
-      </c>
-      <c r="B45" t="s">
-        <v>102</v>
-      </c>
-      <c r="D45" t="s">
-        <v>102</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B45">
+        <v>3</v>
       </c>
       <c r="E45">
         <v>0.66944444179534912</v>
@@ -2798,18 +1983,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M45" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>103</v>
-      </c>
-      <c r="B46" t="s">
-        <v>104</v>
-      </c>
-      <c r="D46" t="s">
-        <v>104</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B46">
+        <v>3</v>
       </c>
       <c r="E46">
         <v>0.74762886762619019</v>
@@ -2836,18 +2015,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M46" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>105</v>
-      </c>
-      <c r="B47" t="s">
-        <v>106</v>
-      </c>
-      <c r="D47" t="s">
-        <v>106</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <v>3</v>
       </c>
       <c r="E47">
         <v>0.67752689123153687</v>
@@ -2874,18 +2047,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M47" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>107</v>
-      </c>
-      <c r="B48" t="s">
-        <v>108</v>
-      </c>
-      <c r="D48" t="s">
-        <v>108</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B48">
+        <v>3</v>
       </c>
       <c r="E48">
         <v>0.66052538156509399</v>
@@ -2912,18 +2079,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M48" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>109</v>
-      </c>
-      <c r="B49" t="s">
-        <v>110</v>
-      </c>
-      <c r="D49" t="s">
-        <v>110</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B49">
+        <v>3</v>
       </c>
       <c r="E49">
         <v>0.57294487953186035</v>
@@ -2950,18 +2111,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>111</v>
-      </c>
-      <c r="B50" t="s">
-        <v>112</v>
-      </c>
-      <c r="D50" t="s">
-        <v>112</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B50">
+        <v>3</v>
       </c>
       <c r="E50">
         <v>0.69018644094467163</v>
@@ -2988,22 +2143,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M50" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>113</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="C51">
         <v>1</v>
       </c>
-      <c r="D51" t="s">
-        <v>115</v>
-      </c>
       <c r="E51">
         <v>0.84276449680328369</v>
       </c>
@@ -3029,22 +2178,16 @@
         <v>200</v>
       </c>
       <c r="M51" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>116</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B52">
         <v>4</v>
       </c>
       <c r="C52">
         <v>2</v>
       </c>
-      <c r="D52" t="s">
-        <v>117</v>
-      </c>
       <c r="E52">
         <v>0.66242587566375732</v>
       </c>
@@ -3070,18 +2213,12 @@
         <v>200</v>
       </c>
       <c r="M52" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>118</v>
-      </c>
-      <c r="B53" t="s">
-        <v>119</v>
-      </c>
-      <c r="D53" t="s">
-        <v>119</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B53">
+        <v>4</v>
       </c>
       <c r="E53">
         <v>0.61060923337936401</v>
@@ -3108,18 +2245,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M53" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>120</v>
-      </c>
-      <c r="B54" t="s">
-        <v>121</v>
-      </c>
-      <c r="D54" t="s">
-        <v>121</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B54">
+        <v>4</v>
       </c>
       <c r="E54">
         <v>0.74880105257034302</v>
@@ -3146,18 +2277,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M54" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>122</v>
-      </c>
-      <c r="B55" t="s">
-        <v>123</v>
-      </c>
-      <c r="D55" t="s">
-        <v>123</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B55">
+        <v>4</v>
       </c>
       <c r="E55">
         <v>0.65678232908248901</v>
@@ -3184,18 +2309,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M55" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>124</v>
-      </c>
-      <c r="B56" t="s">
-        <v>125</v>
-      </c>
-      <c r="D56" t="s">
-        <v>125</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B56">
+        <v>4</v>
       </c>
       <c r="E56">
         <v>0.44597154855728149</v>
@@ -3222,18 +2341,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M56" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>126</v>
-      </c>
-      <c r="B57" t="s">
-        <v>127</v>
-      </c>
-      <c r="D57" t="s">
-        <v>127</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B57">
+        <v>4</v>
       </c>
       <c r="E57">
         <v>0.5798267126083374</v>
@@ -3260,18 +2373,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M57" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>128</v>
-      </c>
-      <c r="B58" t="s">
-        <v>129</v>
-      </c>
-      <c r="D58" t="s">
-        <v>129</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B58">
+        <v>4</v>
       </c>
       <c r="E58">
         <v>0.81914520263671875</v>
@@ -3298,18 +2405,12 @@
         <v>200</v>
       </c>
       <c r="M58" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>130</v>
-      </c>
-      <c r="B59" t="s">
-        <v>131</v>
-      </c>
-      <c r="D59" t="s">
-        <v>131</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B59">
+        <v>4</v>
       </c>
       <c r="E59">
         <v>0.79886859655380249</v>
@@ -3336,18 +2437,12 @@
         <v>200</v>
       </c>
       <c r="M59" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>132</v>
-      </c>
-      <c r="B60" t="s">
-        <v>133</v>
-      </c>
-      <c r="D60" t="s">
-        <v>133</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B60">
+        <v>4</v>
       </c>
       <c r="E60">
         <v>0.93908220529556274</v>
@@ -3374,18 +2469,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M60" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>134</v>
-      </c>
-      <c r="B61" t="s">
-        <v>135</v>
-      </c>
-      <c r="D61" t="s">
-        <v>135</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B61">
+        <v>4</v>
       </c>
       <c r="E61">
         <v>0.69010591506958008</v>
@@ -3412,18 +2501,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M61" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>136</v>
-      </c>
-      <c r="B62" t="s">
-        <v>137</v>
-      </c>
-      <c r="D62" t="s">
-        <v>137</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B62">
+        <v>4</v>
       </c>
       <c r="E62">
         <v>0.67796504497528076</v>
@@ -3450,22 +2533,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M62" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>138</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="C63">
         <v>3</v>
       </c>
-      <c r="D63" t="s">
-        <v>139</v>
-      </c>
       <c r="E63">
         <v>0.76480108499526978</v>
       </c>
@@ -3491,22 +2568,16 @@
         <v>200</v>
       </c>
       <c r="M63" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>140</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="C64">
         <v>4</v>
       </c>
-      <c r="D64" t="s">
-        <v>141</v>
-      </c>
       <c r="E64">
         <v>0.74942934513092041</v>
       </c>
@@ -3532,22 +2603,16 @@
         <v>200</v>
       </c>
       <c r="M64" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>142</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="C65">
         <v>5</v>
       </c>
-      <c r="D65" t="s">
-        <v>143</v>
-      </c>
       <c r="E65">
         <v>0.86284178495407104</v>
       </c>
@@ -3573,22 +2638,16 @@
         <v>200</v>
       </c>
       <c r="M65" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>144</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
-      <c r="D66" t="s">
-        <v>146</v>
-      </c>
       <c r="E66">
         <v>0.73290723562240601</v>
       </c>
@@ -3614,22 +2673,16 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M66" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>147</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C67">
         <v>2</v>
       </c>
-      <c r="D67" t="s">
-        <v>148</v>
-      </c>
       <c r="E67">
         <v>0.70988506078720093</v>
       </c>
@@ -3655,22 +2708,16 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M67" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>149</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C68">
         <v>3</v>
       </c>
-      <c r="D68" t="s">
-        <v>150</v>
-      </c>
       <c r="E68">
         <v>0.94926232099533081</v>
       </c>
@@ -3696,22 +2743,16 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M68" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>151</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C69">
         <v>4</v>
       </c>
-      <c r="D69" t="s">
-        <v>152</v>
-      </c>
       <c r="E69">
         <v>0.72411853075027466</v>
       </c>
@@ -3737,22 +2778,16 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M69" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>153</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C70">
         <v>5</v>
       </c>
-      <c r="D70" t="s">
-        <v>154</v>
-      </c>
       <c r="E70">
         <v>0.75415635108947754</v>
       </c>
@@ -3778,18 +2813,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M70" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>155</v>
-      </c>
-      <c r="B71" t="s">
-        <v>156</v>
-      </c>
-      <c r="D71" t="s">
-        <v>156</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B71">
+        <v>5</v>
       </c>
       <c r="E71">
         <v>0.94449430704116821</v>
@@ -3816,18 +2845,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M71" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>157</v>
-      </c>
-      <c r="B72" t="s">
-        <v>158</v>
-      </c>
-      <c r="D72" t="s">
-        <v>158</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B72">
+        <v>5</v>
       </c>
       <c r="E72">
         <v>0.7880101203918457</v>
@@ -3854,18 +2877,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M72" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>159</v>
-      </c>
-      <c r="B73" t="s">
-        <v>160</v>
-      </c>
-      <c r="D73" t="s">
-        <v>160</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B73">
+        <v>5</v>
       </c>
       <c r="E73">
         <v>0.78574997186660767</v>
@@ -3892,18 +2909,12 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M73" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>161</v>
-      </c>
-      <c r="B74" t="s">
-        <v>162</v>
-      </c>
-      <c r="D74" t="s">
-        <v>162</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B74">
+        <v>5</v>
       </c>
       <c r="E74">
         <v>0.77242547273635864</v>
@@ -3930,18 +2941,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M74" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>163</v>
-      </c>
-      <c r="B75" t="s">
-        <v>164</v>
-      </c>
-      <c r="D75" t="s">
-        <v>164</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B75">
+        <v>5</v>
       </c>
       <c r="E75">
         <v>0.77656018733978271</v>
@@ -3968,18 +2973,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M75" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>165</v>
-      </c>
-      <c r="B76" t="s">
-        <v>166</v>
-      </c>
-      <c r="D76" t="s">
-        <v>166</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B76">
+        <v>5</v>
       </c>
       <c r="E76">
         <v>0.72209632396697998</v>
@@ -4006,18 +3005,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M76" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>167</v>
-      </c>
-      <c r="B77" t="s">
-        <v>168</v>
-      </c>
-      <c r="D77" t="s">
-        <v>168</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B77">
+        <v>5</v>
       </c>
       <c r="E77">
         <v>0.63622087240219116</v>
@@ -4044,18 +3037,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M77" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>169</v>
-      </c>
-      <c r="B78" t="s">
-        <v>170</v>
-      </c>
-      <c r="D78" t="s">
-        <v>170</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B78">
+        <v>5</v>
       </c>
       <c r="E78">
         <v>0.49230161309242249</v>
@@ -4082,18 +3069,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M78" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>171</v>
-      </c>
-      <c r="B79" t="s">
-        <v>172</v>
-      </c>
-      <c r="D79" t="s">
-        <v>172</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B79">
+        <v>5</v>
       </c>
       <c r="E79">
         <v>0.55253821611404419</v>
@@ -4120,22 +3101,16 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M79" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>173</v>
-      </c>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
-      <c r="D80" t="s">
-        <v>175</v>
-      </c>
       <c r="E80">
         <v>0.61885178089141846</v>
       </c>
@@ -4161,22 +3136,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M80" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>176</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
       <c r="C81">
         <v>2</v>
       </c>
-      <c r="D81" t="s">
-        <v>177</v>
-      </c>
       <c r="E81">
         <v>0.65170150995254517</v>
       </c>
@@ -4202,22 +3171,16 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M81" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>178</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
       <c r="C82">
         <v>3</v>
       </c>
-      <c r="D82" t="s">
-        <v>179</v>
-      </c>
       <c r="E82">
         <v>0.73112756013870239</v>
       </c>
@@ -4243,22 +3206,16 @@
         <v>200</v>
       </c>
       <c r="M82" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>180</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
       <c r="C83">
         <v>4</v>
       </c>
-      <c r="D83" t="s">
-        <v>181</v>
-      </c>
       <c r="E83">
         <v>0.606769859790802</v>
       </c>
@@ -4284,22 +3241,16 @@
         <v>200</v>
       </c>
       <c r="M83" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>182</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
       <c r="C84">
         <v>5</v>
       </c>
-      <c r="D84" t="s">
-        <v>183</v>
-      </c>
       <c r="E84">
         <v>0.58059161901473999</v>
       </c>
@@ -4325,18 +3276,12 @@
         <v>193.33333333333329</v>
       </c>
       <c r="M84" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>184</v>
-      </c>
-      <c r="B85" t="s">
-        <v>185</v>
-      </c>
-      <c r="D85" t="s">
-        <v>185</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B85">
+        <v>6</v>
       </c>
       <c r="E85">
         <v>0.64421916007995605</v>
@@ -4363,18 +3308,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M85" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>186</v>
-      </c>
-      <c r="B86" t="s">
-        <v>187</v>
-      </c>
-      <c r="D86" t="s">
-        <v>187</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B86">
+        <v>6</v>
       </c>
       <c r="E86">
         <v>0.65695476531982422</v>
@@ -4401,18 +3340,12 @@
         <v>190</v>
       </c>
       <c r="M86" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>188</v>
-      </c>
-      <c r="B87" t="s">
-        <v>189</v>
-      </c>
-      <c r="D87" t="s">
-        <v>189</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B87">
+        <v>6</v>
       </c>
       <c r="E87">
         <v>0.61346125602722168</v>
@@ -4439,18 +3372,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M87" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>190</v>
-      </c>
-      <c r="B88" t="s">
-        <v>191</v>
-      </c>
-      <c r="D88" t="s">
-        <v>191</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B88">
+        <v>6</v>
       </c>
       <c r="E88">
         <v>0.60480892658233643</v>
@@ -4477,18 +3404,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M88" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>192</v>
-      </c>
-      <c r="B89" t="s">
-        <v>193</v>
-      </c>
-      <c r="D89" t="s">
-        <v>193</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B89">
+        <v>6</v>
       </c>
       <c r="E89">
         <v>0.59211194515228271</v>
@@ -4515,18 +3436,12 @@
         <v>180</v>
       </c>
       <c r="M89" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>194</v>
-      </c>
-      <c r="B90" t="s">
-        <v>195</v>
-      </c>
-      <c r="D90" t="s">
-        <v>195</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="90" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B90">
+        <v>6</v>
       </c>
       <c r="E90">
         <v>0.76281583309173584</v>
@@ -4553,18 +3468,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M90" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>196</v>
-      </c>
-      <c r="B91" t="s">
-        <v>197</v>
-      </c>
-      <c r="D91" t="s">
-        <v>197</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B91">
+        <v>6</v>
       </c>
       <c r="E91">
         <v>0.7515333890914917</v>
@@ -4591,18 +3500,12 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M91" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>198</v>
-      </c>
-      <c r="B92" t="s">
-        <v>199</v>
-      </c>
-      <c r="D92" t="s">
-        <v>199</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="92" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B92">
+        <v>6</v>
       </c>
       <c r="E92">
         <v>0.5477796196937561</v>
@@ -4629,18 +3532,12 @@
         <v>200</v>
       </c>
       <c r="M92" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>200</v>
-      </c>
-      <c r="B93" t="s">
-        <v>201</v>
-      </c>
-      <c r="D93" t="s">
-        <v>201</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="93" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B93">
+        <v>6</v>
       </c>
       <c r="E93">
         <v>0.63564527034759521</v>
@@ -4667,18 +3564,12 @@
         <v>203.33333333333329</v>
       </c>
       <c r="M93" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>202</v>
-      </c>
-      <c r="B94" t="s">
-        <v>203</v>
-      </c>
-      <c r="D94" t="s">
-        <v>203</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B94">
+        <v>6</v>
       </c>
       <c r="E94">
         <v>0.59530627727508545</v>
@@ -4705,22 +3596,16 @@
         <v>206.66666666666671</v>
       </c>
       <c r="M94" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>204</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
-        <v>205</v>
+        <v>17</v>
       </c>
       <c r="C95">
         <v>1</v>
       </c>
-      <c r="D95" t="s">
-        <v>206</v>
-      </c>
       <c r="E95">
         <v>0.38947203755378718</v>
       </c>
@@ -4746,22 +3631,16 @@
         <v>140</v>
       </c>
       <c r="M95" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>207</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="96" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
-        <v>205</v>
+        <v>17</v>
       </c>
       <c r="C96">
         <v>2</v>
       </c>
-      <c r="D96" t="s">
-        <v>208</v>
-      </c>
       <c r="E96">
         <v>0.36370760202407842</v>
       </c>
@@ -4787,22 +3666,16 @@
         <v>120</v>
       </c>
       <c r="M96" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>209</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="97" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
-        <v>210</v>
+        <v>18</v>
       </c>
       <c r="C97">
         <v>1</v>
       </c>
-      <c r="D97" t="s">
-        <v>211</v>
-      </c>
       <c r="E97">
         <v>0.2409983575344086</v>
       </c>
@@ -4828,21 +3701,15 @@
         <v>120</v>
       </c>
       <c r="M97" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>212</v>
-      </c>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="98" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
-        <v>213</v>
+        <v>19</v>
       </c>
       <c r="C98" t="s">
-        <v>214</v>
-      </c>
-      <c r="D98" t="s">
-        <v>215</v>
+        <v>20</v>
       </c>
       <c r="E98">
         <v>0.79560792446136475</v>
@@ -4869,7 +3736,7 @@
         <v>196.66666666666671</v>
       </c>
       <c r="M98" t="s">
-        <v>73</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>